<commit_message>
Repair VcScHv domain behavior, typed interfaces and independent tests
</commit_message>
<xml_diff>
--- a/Documentation/VcScHv_26R1_变更记录.xlsx
+++ b/Documentation/VcScHv_26R1_变更记录.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R4927008444bd4f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25R3" sheetId="2" r:id="Rb84321c05b454240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26R1" sheetId="3" r:id="Rda8cde116bb24f5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rabffd1c5453c475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25R3" sheetId="2" r:id="R3da8c6cce2ff4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26R1" sheetId="3" r:id="Rc133652086024bc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +53,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -67,6 +67,15 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -303,7 +312,7 @@
         <x:v>Current version</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>11.2.1_0</x:v>
+        <x:v>12.0.0_0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -447,92 +456,94 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>模型版本</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>变更ID</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>问题ID</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>需求ID</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>需求文件</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>需求文件版本</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>更改部分所处位置</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>更改部分原逻辑</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="6" t="str">
         <x:v>更改后的逻辑</x:v>
       </x:c>
-      <x:c r="K1" s="4" t="str">
+      <x:c r="K1" s="6" t="str">
         <x:v>变更原因</x:v>
       </x:c>
-      <x:c r="L1" s="4" t="str">
+      <x:c r="L1" s="6" t="str">
         <x:v>变更原因详细说明</x:v>
       </x:c>
-      <x:c r="M1" s="4" t="str">
+      <x:c r="M1" s="6" t="str">
         <x:v>模型负责人</x:v>
       </x:c>
-      <x:c r="N1" s="4" t="str">
+      <x:c r="N1" s="6" t="str">
         <x:v>软件设计需求负责人</x:v>
       </x:c>
-      <x:c r="O1" s="4" t="str">
+      <x:c r="O1" s="6" t="str">
         <x:v>系统需求负责人</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="100" customHeight="1">
-      <x:c r="A2" s="5" t="n">
+    <x:row r="2" ht="150" customHeight="1">
+      <x:c r="A2" s="7" t="n">
         <x:v>46275</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="str">
-        <x:v>11.2.1_0</x:v>
-      </x:c>
-      <x:c r="C2" s="2" t="str">
-        <x:v>NEP-11-CHG-002</x:v>
-      </x:c>
-      <x:c r="D2" s="2"/>
-      <x:c r="E2" s="2" t="str">
+      <x:c r="B2" s="8" t="str">
+        <x:v>12.0.0_0</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>NEP-11-CHG-003</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>NEP-11-REPAIR</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
         <x:v>NEP-11-004</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="str">
-        <x:v>Requirements.txt</x:v>
-      </x:c>
-      <x:c r="G2" s="2" t="str">
-        <x:v>1.1</x:v>
-      </x:c>
-      <x:c r="H2" s="2" t="str">
-        <x:v>VcScHv/BusinessDecision</x:v>
-      </x:c>
-      <x:c r="I2" s="2" t="str">
-        <x:v>Instantaneous command only; no domain state</x:v>
-      </x:c>
-      <x:c r="J2" s="2" t="str">
-        <x:v>Stateful high_voltage_sequence; explicit reset, transition and recovery behavior</x:v>
-      </x:c>
-      <x:c r="K2" s="2" t="str">
-        <x:v>Business realism and interface correction</x:v>
-      </x:c>
-      <x:c r="L2" s="2" t="str">
-        <x:v>Root signals added: 0; root signals removed: 0. TargetSoc unit corrected to percent for charging. Baseline and current SLX snapshots retained outside candidate. Patch 11.2.1 normalizes reset through a library component and gates selected engineering conversions by qualification; output behavior remains equivalent over recorded scenarios.</x:v>
-      </x:c>
-      <x:c r="M2" s="2" t="str">
+      <x:c r="F2" s="8" t="str">
+        <x:v>BusinessBehavior.md; InterfaceChanges.json</x:v>
+      </x:c>
+      <x:c r="G2" s="8" t="str">
+        <x:v>2.0</x:v>
+      </x:c>
+      <x:c r="H2" s="8" t="str">
+        <x:v>VcScHv/BusinessDecision; root IN/OUT and signal qualification</x:v>
+      </x:c>
+      <x:c r="I2" s="8" t="str">
+        <x:v>Floating elapsed timer tested completion before the late timeout boundary.</x:v>
+      </x:c>
+      <x:c r="J2" s="8" t="str">
+        <x:v>Integer tick precharge deadline: 490/500 ms success, 510 ms rejected; low voltage cannot close.</x:v>
+      </x:c>
+      <x:c r="K2" s="8" t="str">
+        <x:v>Business behavior and typed interface repair</x:v>
+      </x:c>
+      <x:c r="L2" s="8" t="str">
+        <x:v>Root signals added: 3; removed: 0; type/unit/range changes: 36. Exact names and before/after values: InterfaceChanges.json. Baseline 11.2.1_0 -&gt; 12.0.0_0; original snapshot retained in Git parent.</x:v>
+      </x:c>
+      <x:c r="M2" s="8" t="str">
         <x:v>Synthetic model maintainer</x:v>
       </x:c>
-      <x:c r="N2" s="2"/>
-      <x:c r="O2" s="2"/>
+      <x:c r="N2" s="8"/>
+      <x:c r="O2" s="8"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Repair engineering interfaces, calibration use and executable test records
</commit_message>
<xml_diff>
--- a/Documentation/VcScHv_26R1_变更记录.xlsx
+++ b/Documentation/VcScHv_26R1_变更记录.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rabffd1c5453c475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25R3" sheetId="2" r:id="R3da8c6cce2ff4a39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26R1" sheetId="3" r:id="Rc133652086024bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R08359b2e21fc469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25R3" sheetId="2" r:id="R2179da0e011e43a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26R1" sheetId="3" r:id="R5cb7bae152da43c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -545,6 +545,49 @@
       <x:c r="N2" s="8"/>
       <x:c r="O2" s="8"/>
     </x:row>
+    <x:row r="3" ht="150" customHeight="1">
+      <x:c r="A3" s="7" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>12.0.0_0</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>NEP-11-CHG-004</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="str">
+        <x:v>NEP-11-FIDELITY-REPAIR</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="str">
+        <x:v>NEP-11-ENGINEERING</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="str">
+        <x:v>EngineeringRepair.json; BusinessBehavior.md</x:v>
+      </x:c>
+      <x:c r="G3" s="8" t="str">
+        <x:v>3.0</x:v>
+      </x:c>
+      <x:c r="H3" s="8" t="str">
+        <x:v>Model; Src LAB where present; UnitTest/UintTest SWUT</x:v>
+      </x:c>
+      <x:c r="I3" s="8" t="str">
+        <x:v>See repair findings and Git parent for module-specific baseline.</x:v>
+      </x:c>
+      <x:c r="J3" s="8" t="str">
+        <x:v>0 compacted channels; 0 added calibration objects; property-specific SWUT tolerance and exact stimulus rows.</x:v>
+      </x:c>
+      <x:c r="K3" s="8" t="str">
+        <x:v>Source-grounded engineering repair</x:v>
+      </x:c>
+      <x:c r="L3" s="8" t="str">
+        <x:v>Actual consumers and shapes in EngineeringRepair.json. Existing root interfaces retained. Local synthetic calibration; no physical ECU or recovered internal algorithm claim.</x:v>
+      </x:c>
+      <x:c r="M3" s="8" t="str">
+        <x:v>Synthetic model maintainer</x:v>
+      </x:c>
+      <x:c r="N3" s="8"/>
+      <x:c r="O3" s="8"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>